<commit_message>
contact test case automation
contact test case automation
format test cases excel
</commit_message>
<xml_diff>
--- a/Test case sheet/Test cases For Practice.xlsx
+++ b/Test case sheet/Test cases For Practice.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Swag-Labs-test-cases-and-Automation-code\Test case sheet\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CD9EAC3-6C5C-4109-A5E2-A941803F9B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Swag Labs" sheetId="1" r:id="rId5"/>
+    <sheet name="Swag Labs" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -83,18 +92,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -120,18 +131,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -157,18 +170,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -190,18 +205,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -226,18 +243,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -263,18 +282,20 @@
   <si>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t xml:space="preserve">https://www.saucedemo.com
 </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
         <rFont val="Arial"/>
-        <color rgb="FF1F1F1F"/>
-        <u/>
       </rPr>
       <t>username: standard_user
 password: secrect_sauce</t>
@@ -363,15 +384,17 @@
   <si>
     <r>
       <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
       </rPr>
       <t xml:space="preserve">Redirected to </t>
     </r>
     <r>
       <rPr>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
       </rPr>
       <t>https://saucelabs.com</t>
     </r>
@@ -640,34 +663,45 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
-  </numFmts>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -676,7 +710,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -686,7 +720,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -700,70 +740,53 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="13">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -953,29 +976,36 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="22.63"/>
-    <col customWidth="1" min="3" max="3" width="38.0"/>
-    <col customWidth="1" min="4" max="4" width="63.0"/>
-    <col customWidth="1" min="5" max="5" width="44.88"/>
-    <col customWidth="1" min="6" max="6" width="22.25"/>
-    <col customWidth="1" min="7" max="7" width="68.0"/>
-    <col customWidth="1" min="9" max="9" width="13.88"/>
+    <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="65.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="72" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="75.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="10"/>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
@@ -987,12 +1017,13 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
+      <c r="B2" s="10"/>
       <c r="C2" s="2">
-        <v>46191.0</v>
+        <v>46191</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1002,10 +1033,11 @@
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>3</v>
       </c>
+      <c r="B3" s="10"/>
       <c r="C3" s="3" t="s">
         <v>4</v>
       </c>
@@ -1017,10 +1049,11 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
+      <c r="B4" s="10"/>
       <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
@@ -1032,7 +1065,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -1064,671 +1097,671 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:10" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="9"/>
-    </row>
-    <row r="7">
+      <c r="H6" s="5"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" spans="1:10" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="9"/>
-    </row>
-    <row r="8">
+      <c r="H7" s="5"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="5"/>
+    </row>
+    <row r="8" spans="1:10" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="9"/>
-    </row>
-    <row r="9">
+      <c r="H8" s="5"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="9"/>
-    </row>
-    <row r="10">
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="5"/>
+    </row>
+    <row r="10" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="9"/>
-    </row>
-    <row r="11">
+      <c r="H10" s="5"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="5"/>
+    </row>
+    <row r="11" spans="1:10" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="9"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="9"/>
-    </row>
-    <row r="12">
+      <c r="H11" s="5"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="5"/>
+    </row>
+    <row r="12" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10" t="s">
+      <c r="F12" s="5"/>
+      <c r="G12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H12" s="9"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="9"/>
-    </row>
-    <row r="13">
+      <c r="H12" s="5"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="5"/>
+    </row>
+    <row r="13" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="10" t="s">
+      <c r="F13" s="5"/>
+      <c r="G13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H13" s="9"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="9"/>
-    </row>
-    <row r="14">
+      <c r="H13" s="5"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="5"/>
+    </row>
+    <row r="14" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="7" t="s">
+      <c r="F14" s="5"/>
+      <c r="G14" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H14" s="9"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15">
+      <c r="H14" s="5"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="5"/>
+    </row>
+    <row r="15" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="F15" s="6"/>
-      <c r="G15" s="10" t="s">
+      <c r="F15" s="5"/>
+      <c r="G15" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="H15" s="9"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="9"/>
-    </row>
-    <row r="16">
+      <c r="H15" s="5"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="5"/>
+    </row>
+    <row r="16" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="F16" s="9"/>
-      <c r="G16" s="13" t="s">
+      <c r="F16" s="5"/>
+      <c r="G16" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="9"/>
-    </row>
-    <row r="17">
+      <c r="H16" s="5"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="7" t="s">
+      <c r="F17" s="5"/>
+      <c r="G17" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="H17" s="9"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="9"/>
-    </row>
-    <row r="18">
+      <c r="H17" s="5"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="5"/>
+    </row>
+    <row r="18" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="10" t="s">
+      <c r="F18" s="5"/>
+      <c r="G18" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="H18" s="9"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="9"/>
-    </row>
-    <row r="19">
+      <c r="H18" s="5"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="5"/>
+    </row>
+    <row r="19" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="10" t="s">
+      <c r="F19" s="5"/>
+      <c r="G19" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H19" s="9"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="9"/>
-    </row>
-    <row r="20">
+      <c r="H19" s="5"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="7" t="s">
+      <c r="F20" s="5"/>
+      <c r="G20" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="H20" s="9"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="9"/>
-    </row>
-    <row r="21">
+      <c r="H20" s="5"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="10" t="s">
+      <c r="F21" s="5"/>
+      <c r="G21" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="H21" s="9"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="9"/>
-    </row>
-    <row r="22">
+      <c r="H21" s="5"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="7" t="s">
+      <c r="C22" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="F22" s="9"/>
-      <c r="G22" s="7" t="s">
+      <c r="F22" s="5"/>
+      <c r="G22" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="H22" s="9"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23">
+      <c r="H22" s="5"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="5"/>
+    </row>
+    <row r="23" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F23" s="9"/>
-      <c r="G23" s="11" t="s">
+      <c r="F23" s="5"/>
+      <c r="G23" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="9"/>
-    </row>
-    <row r="24">
+      <c r="H23" s="5"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="5"/>
+    </row>
+    <row r="24" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="F24" s="9"/>
-      <c r="G24" s="7" t="s">
+      <c r="F24" s="5"/>
+      <c r="G24" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="H24" s="9"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="9"/>
-    </row>
-    <row r="25">
+      <c r="H24" s="5"/>
+      <c r="I24" s="6"/>
+      <c r="J24" s="5"/>
+    </row>
+    <row r="25" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="5" t="s">
         <v>121</v>
       </c>
       <c r="E25" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="F25" s="9"/>
-      <c r="G25" s="6" t="s">
+      <c r="F25" s="5"/>
+      <c r="G25" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="H25" s="9"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26">
+      <c r="H25" s="5"/>
+      <c r="I25" s="6"/>
+      <c r="J25" s="5"/>
+    </row>
+    <row r="26" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="5" t="s">
         <v>126</v>
       </c>
       <c r="E26" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="F26" s="9"/>
-      <c r="G26" s="6" t="s">
+      <c r="F26" s="5"/>
+      <c r="G26" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="H26" s="9"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27">
+      <c r="H26" s="5"/>
+      <c r="I26" s="6"/>
+      <c r="J26" s="5"/>
+    </row>
+    <row r="27" spans="1:10" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="6" t="s">
+      <c r="F27" s="5"/>
+      <c r="G27" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="H27" s="9"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="9"/>
-    </row>
-    <row r="28">
+      <c r="H27" s="5"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="5"/>
+    </row>
+    <row r="28" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="F28" s="9"/>
-      <c r="G28" s="12" t="s">
+      <c r="F28" s="5"/>
+      <c r="G28" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="H28" s="9"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="9"/>
-    </row>
-    <row r="29">
+      <c r="H28" s="5"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="5"/>
+    </row>
+    <row r="29" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="F29" s="9"/>
-      <c r="G29" s="6" t="s">
+      <c r="F29" s="5"/>
+      <c r="G29" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="H29" s="9"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="9"/>
-    </row>
-    <row r="30">
+      <c r="H29" s="5"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="5"/>
+    </row>
+    <row r="30" spans="1:10" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="F30" s="9"/>
-      <c r="G30" s="6" t="s">
+      <c r="F30" s="5"/>
+      <c r="G30" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="9"/>
-    </row>
-    <row r="31">
+      <c r="H30" s="5"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="5"/>
+    </row>
+    <row r="31" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="F31" s="9"/>
-      <c r="G31" s="6" t="s">
+      <c r="F31" s="5"/>
+      <c r="G31" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="9"/>
-    </row>
-    <row r="32">
+      <c r="H31" s="5"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="5"/>
+    </row>
+    <row r="32" spans="1:10" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="F32" s="9"/>
-      <c r="G32" s="6" t="s">
+      <c r="F32" s="5"/>
+      <c r="G32" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="H32" s="9"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="9"/>
-    </row>
-    <row r="33">
+      <c r="H32" s="5"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="5"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
       <c r="E33" s="1"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -1736,11 +1769,11 @@
       <c r="E34" s="1"/>
       <c r="G34" s="1"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
       <c r="E35" s="1"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -1748,11 +1781,11 @@
       <c r="E36" s="1"/>
       <c r="G36" s="1"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="E37" s="1"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -1760,11 +1793,11 @@
       <c r="E38" s="1"/>
       <c r="G38" s="1"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
       <c r="E39" s="1"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
@@ -1772,7 +1805,7 @@
       <c r="E40" s="1"/>
       <c r="G40" s="1"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
@@ -1780,11 +1813,11 @@
       <c r="E41" s="1"/>
       <c r="G41" s="1"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
@@ -1792,12 +1825,12 @@
       <c r="E43" s="1"/>
       <c r="G43" s="1"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
     </row>
@@ -1808,20 +1841,20 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
   </mergeCells>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I32">
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="I6:I32" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail,Error"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="F6"/>
-    <hyperlink r:id="rId2" ref="F7"/>
-    <hyperlink r:id="rId3" ref="F8"/>
-    <hyperlink r:id="rId4" ref="F9"/>
-    <hyperlink r:id="rId5" ref="F10"/>
-    <hyperlink r:id="rId6" ref="F11"/>
-    <hyperlink r:id="rId7" ref="G16"/>
+    <hyperlink ref="F6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="F7" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="F8" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="F9" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="F10" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="F11" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="G16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
   </hyperlinks>
-  <drawing r:id="rId8"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>